<commit_message>
docs: Minor changes on Docs
</commit_message>
<xml_diff>
--- a/Design/BusMatrix.xlsx
+++ b/Design/BusMatrix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Github\hospital-data-warehouse\Design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F03DDE9A-F0DA-4E08-B184-F07FBE6C1B58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1A951C1-D3A6-4344-8C20-59A8C2A8020E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="2745" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{50652A4D-B507-3747-9A78-47BC79B2AC43}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{50652A4D-B507-3747-9A78-47BC79B2AC43}"/>
   </bookViews>
   <sheets>
     <sheet name="Bus Matrix" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="28">
   <si>
     <t>Business Processes</t>
   </si>
@@ -94,9 +94,6 @@
     <t>Patient</t>
   </si>
   <si>
-    <t>Caregiver</t>
-  </si>
-  <si>
     <t>Diagnosis</t>
   </si>
   <si>
@@ -115,12 +112,6 @@
     <t>Operational Events</t>
   </si>
   <si>
-    <t>Discharge Callout</t>
-  </si>
-  <si>
-    <t>Service Timeline</t>
-  </si>
-  <si>
     <t>Patient Output</t>
   </si>
   <si>
@@ -130,7 +121,7 @@
     <t>Facility Utilization</t>
   </si>
   <si>
-    <t>Measurement Type</t>
+    <t>Lab Items</t>
   </si>
 </sst>
 </file>
@@ -310,7 +301,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -332,52 +323,49 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -703,17 +691,17 @@
   </cols>
   <sheetData>
     <row r="10" spans="6:15" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="G10" s="13" t="s">
+      <c r="G10" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="H10" s="13"/>
-      <c r="I10" s="13"/>
-      <c r="J10" s="13"/>
-      <c r="K10" s="13"/>
-      <c r="L10" s="13"/>
-      <c r="M10" s="13"/>
-      <c r="N10" s="13"/>
-      <c r="O10" s="13"/>
+      <c r="H10" s="14"/>
+      <c r="I10" s="14"/>
+      <c r="J10" s="14"/>
+      <c r="K10" s="14"/>
+      <c r="L10" s="14"/>
+      <c r="M10" s="14"/>
+      <c r="N10" s="14"/>
+      <c r="O10" s="14"/>
     </row>
     <row r="11" spans="6:15" ht="64.5" x14ac:dyDescent="0.4">
       <c r="F11" s="2" t="s">
@@ -881,168 +869,157 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C046CFE-F1E5-9B43-8470-62B2AC7A197C}">
-  <dimension ref="B1:AC23"/>
+  <dimension ref="B1:AB21"/>
   <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="2" customWidth="1"/>
     <col min="4" max="4" width="7.69921875" customWidth="1"/>
     <col min="5" max="5" width="12.09765625" hidden="1" customWidth="1"/>
-    <col min="6" max="29" width="3.59765625" bestFit="1" customWidth="1"/>
+    <col min="6" max="28" width="3.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:29" ht="96.75" x14ac:dyDescent="0.3">
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="12" t="s">
+    <row r="1" spans="2:28" ht="49.5" x14ac:dyDescent="0.3">
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="H1" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="I1" s="12" t="s">
+      <c r="H1" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="I1" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="J1" s="11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="2:28" x14ac:dyDescent="0.3">
+      <c r="B2" s="23" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="23"/>
+    </row>
+    <row r="3" spans="2:28" x14ac:dyDescent="0.3">
+      <c r="B3" s="8"/>
+      <c r="C3" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J3" s="9"/>
+    </row>
+    <row r="4" spans="2:28" x14ac:dyDescent="0.3">
+      <c r="B4" s="8"/>
+      <c r="C4" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="18"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+    </row>
+    <row r="5" spans="2:28" x14ac:dyDescent="0.3">
+      <c r="B5" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="K1" s="12" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="2:29" x14ac:dyDescent="0.3">
-      <c r="B2" s="18" t="s">
+      <c r="C5" s="21"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="21"/>
+      <c r="H5" s="21"/>
+      <c r="I5" s="21"/>
+      <c r="J5" s="22"/>
+    </row>
+    <row r="6" spans="2:28" x14ac:dyDescent="0.3">
+      <c r="B6" s="8"/>
+      <c r="C6" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="18"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="2:28" x14ac:dyDescent="0.3">
+      <c r="B7" s="8"/>
+      <c r="C7" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
-      <c r="J2" s="18"/>
-      <c r="K2" s="18"/>
-    </row>
-    <row r="3" spans="2:29" x14ac:dyDescent="0.3">
-      <c r="B3" s="8"/>
-      <c r="C3" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="H3" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="I3" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="J3" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="K3" s="9"/>
-    </row>
-    <row r="4" spans="2:29" x14ac:dyDescent="0.3">
-      <c r="B4" s="8"/>
-      <c r="C4" s="20" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" s="21"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="G4" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="H4" s="11"/>
-      <c r="I4" s="11"/>
-      <c r="J4" s="11"/>
-      <c r="K4" s="11"/>
-    </row>
-    <row r="5" spans="2:29" x14ac:dyDescent="0.3">
-      <c r="B5" s="8"/>
-      <c r="C5" s="20" t="s">
-        <v>25</v>
-      </c>
-      <c r="D5" s="21"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="G5" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="H5" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="11"/>
-    </row>
-    <row r="6" spans="2:29" x14ac:dyDescent="0.3">
-      <c r="B6" s="8"/>
-      <c r="C6" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="D6" s="24"/>
-      <c r="E6" s="21"/>
-      <c r="F6" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="9"/>
-    </row>
-    <row r="7" spans="2:29" x14ac:dyDescent="0.3">
-      <c r="B7" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" s="16"/>
-      <c r="D7" s="16"/>
-      <c r="E7" s="16"/>
-      <c r="F7" s="16"/>
-      <c r="G7" s="16"/>
-      <c r="H7" s="16"/>
-      <c r="I7" s="16"/>
-      <c r="J7" s="16"/>
-      <c r="K7" s="17"/>
-    </row>
-    <row r="8" spans="2:29" x14ac:dyDescent="0.3">
+      <c r="D7" s="18"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="H7" s="10"/>
+      <c r="I7" s="10"/>
+      <c r="J7" s="13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="2:28" x14ac:dyDescent="0.3">
       <c r="B8" s="8"/>
-      <c r="C8" s="23" t="s">
+      <c r="C8" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="24"/>
-      <c r="E8" s="21"/>
-      <c r="F8" s="25" t="s">
+      <c r="D8" s="18"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="9" t="s">
         <v>16</v>
       </c>
       <c r="G8" s="9" t="s">
         <v>16</v>
       </c>
       <c r="H8" s="9"/>
-      <c r="I8" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="J8" s="9"/>
-      <c r="K8" s="25" t="s">
-        <v>16</v>
-      </c>
+      <c r="I8" s="9"/>
+      <c r="J8" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="K8" s="6"/>
       <c r="L8" s="6"/>
       <c r="M8" s="6"/>
       <c r="N8" s="6"/>
@@ -1060,160 +1037,103 @@
       <c r="Z8" s="6"/>
       <c r="AA8" s="6"/>
       <c r="AB8" s="6"/>
-      <c r="AC8" s="6"/>
-    </row>
-    <row r="9" spans="2:29" x14ac:dyDescent="0.3">
-      <c r="B9" s="8"/>
-      <c r="C9" s="20" t="s">
-        <v>27</v>
-      </c>
-      <c r="D9" s="24"/>
-      <c r="E9" s="22"/>
-      <c r="F9" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="G9" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="H9" s="11"/>
-      <c r="I9" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="J9" s="11"/>
-      <c r="K9" s="25" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" spans="2:29" x14ac:dyDescent="0.3">
-      <c r="B10" s="8"/>
-      <c r="C10" s="23" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" s="24"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="G10" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
-      <c r="K10" s="25" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="11" spans="2:29" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="2:28" x14ac:dyDescent="0.3">
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+    </row>
+    <row r="10" spans="2:28" x14ac:dyDescent="0.3">
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+    </row>
+    <row r="11" spans="2:28" x14ac:dyDescent="0.3">
       <c r="F11" s="7"/>
       <c r="G11" s="7"/>
       <c r="H11" s="7"/>
       <c r="I11" s="7"/>
       <c r="J11" s="7"/>
-      <c r="K11" s="7"/>
-    </row>
-    <row r="12" spans="2:29" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="2:28" x14ac:dyDescent="0.3">
       <c r="F12" s="7"/>
       <c r="G12" s="7"/>
       <c r="H12" s="7"/>
       <c r="I12" s="7"/>
       <c r="J12" s="7"/>
-      <c r="K12" s="7"/>
-    </row>
-    <row r="13" spans="2:29" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="2:28" x14ac:dyDescent="0.3">
       <c r="F13" s="7"/>
       <c r="G13" s="7"/>
       <c r="H13" s="7"/>
       <c r="I13" s="7"/>
       <c r="J13" s="7"/>
-      <c r="K13" s="7"/>
-    </row>
-    <row r="14" spans="2:29" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="2:28" x14ac:dyDescent="0.3">
       <c r="F14" s="7"/>
       <c r="G14" s="7"/>
       <c r="H14" s="7"/>
       <c r="I14" s="7"/>
       <c r="J14" s="7"/>
-      <c r="K14" s="7"/>
-    </row>
-    <row r="15" spans="2:29" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="2:28" x14ac:dyDescent="0.3">
       <c r="F15" s="7"/>
       <c r="G15" s="7"/>
       <c r="H15" s="7"/>
       <c r="I15" s="7"/>
       <c r="J15" s="7"/>
-      <c r="K15" s="7"/>
-    </row>
-    <row r="16" spans="2:29" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="2:28" x14ac:dyDescent="0.3">
       <c r="F16" s="7"/>
       <c r="G16" s="7"/>
       <c r="H16" s="7"/>
       <c r="I16" s="7"/>
       <c r="J16" s="7"/>
-      <c r="K16" s="7"/>
-    </row>
-    <row r="17" spans="6:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="6:10" x14ac:dyDescent="0.3">
       <c r="F17" s="7"/>
       <c r="G17" s="7"/>
       <c r="H17" s="7"/>
       <c r="I17" s="7"/>
       <c r="J17" s="7"/>
-      <c r="K17" s="7"/>
-    </row>
-    <row r="18" spans="6:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="6:10" x14ac:dyDescent="0.3">
       <c r="F18" s="7"/>
       <c r="G18" s="7"/>
       <c r="H18" s="7"/>
       <c r="I18" s="7"/>
       <c r="J18" s="7"/>
-      <c r="K18" s="7"/>
-    </row>
-    <row r="19" spans="6:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="6:10" x14ac:dyDescent="0.3">
       <c r="F19" s="7"/>
       <c r="G19" s="7"/>
       <c r="H19" s="7"/>
       <c r="I19" s="7"/>
       <c r="J19" s="7"/>
-      <c r="K19" s="7"/>
-    </row>
-    <row r="20" spans="6:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="20" spans="6:10" x14ac:dyDescent="0.3">
       <c r="F20" s="7"/>
       <c r="G20" s="7"/>
       <c r="H20" s="7"/>
       <c r="I20" s="7"/>
       <c r="J20" s="7"/>
-      <c r="K20" s="7"/>
-    </row>
-    <row r="21" spans="6:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="6:10" x14ac:dyDescent="0.3">
       <c r="F21" s="7"/>
-      <c r="G21" s="7"/>
-      <c r="H21" s="7"/>
-      <c r="I21" s="7"/>
-      <c r="J21" s="7"/>
-      <c r="K21" s="7"/>
-    </row>
-    <row r="22" spans="6:11" x14ac:dyDescent="0.3">
-      <c r="F22" s="7"/>
-      <c r="G22" s="7"/>
-      <c r="H22" s="7"/>
-      <c r="I22" s="7"/>
-      <c r="J22" s="7"/>
-      <c r="K22" s="7"/>
-    </row>
-    <row r="23" spans="6:11" x14ac:dyDescent="0.3">
-      <c r="F23" s="7"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="8">
+    <mergeCell ref="C8:E8"/>
+    <mergeCell ref="B5:J5"/>
+    <mergeCell ref="B2:J2"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="C4:E4"/>
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="C8:E8"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="B7:K7"/>
-    <mergeCell ref="B2:K2"/>
-    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="C7:D7"/>
     <mergeCell ref="C6:E6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>